<commit_message>
Ka irgend a update oder so
</commit_message>
<xml_diff>
--- a/D_Descriptions/Risiken.xlsx
+++ b/D_Descriptions/Risiken.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://togetherglobal.sharepoint.com/sites/LTN-educationinstitutioncooperation-HTLDiplomarbeit-3DScanner/Shared Documents/HTL Diplomarbeit - 3D Scanner/Risiken/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\Diplomarbeit\Git\3D_Scanner_New\3D_Scanner\D_Descriptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="294" documentId="11_E45CACB30E60352A828C57A285813AE534ED4106" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C62210F2-ABED-42B5-AE89-3C0DE1532CA4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8E855D-2C29-4AFF-AB2D-8CA830CF4376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Risiken" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="61">
   <si>
     <t>Thema</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Auswirkung</t>
   </si>
   <si>
-    <t>Umsetzung</t>
-  </si>
-  <si>
     <t>Raspberry Pi</t>
   </si>
   <si>
@@ -74,9 +71,6 @@
     <t>Distanzmessung</t>
   </si>
   <si>
-    <t>Die Messung ist zu ungenau bei kleinere Objekten (Tiefenkamera +- 2cm)</t>
-  </si>
-  <si>
     <t>sehr hoch</t>
   </si>
   <si>
@@ -110,9 +104,6 @@
     <t>Benutzer verfälscht das Ergebnis nicht</t>
   </si>
   <si>
-    <t>Buzzer, LED-Leuchten, usw.</t>
-  </si>
-  <si>
     <t>Interface</t>
   </si>
   <si>
@@ -149,12 +140,6 @@
     <t>Es sind keine 4 Schnittstellen für die RPI CAMs vorhanden. Es werden daher nur 2 RPI Cams und zwei USB CAMs verwendet</t>
   </si>
   <si>
-    <t>spezielle LIDAR/TOF Tiefenkamera</t>
-  </si>
-  <si>
-    <t>Besser Auflösende Kamera</t>
-  </si>
-  <si>
     <t>Scanner würde viel länger als mit der micro sd funktionieren. Eine Adapterplatine wäre nötig</t>
   </si>
   <si>
@@ -176,9 +161,6 @@
     <t>Betriebsystem auf einer SSD nmve laufen lassen, da eine micro sd schnell kaputt gehen kann</t>
   </si>
   <si>
-    <t>Wird als Feature zurückgestellt.</t>
-  </si>
-  <si>
     <t>Risikoantwort?</t>
   </si>
   <si>
@@ -212,22 +194,31 @@
     <t>wird so umgesetzt</t>
   </si>
   <si>
-    <t>Es könnte eine vereinfate gerundete zahl mit 0 gramm dargestellt werden</t>
-  </si>
-  <si>
-    <t>0g oder leer oder "nicht erfassbar"</t>
-  </si>
-  <si>
-    <t>0 mm oder "nicht erfassbar"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bei kleinen einträgen wie 1.5 mm wird eine Messung schwierig, daher </t>
-  </si>
-  <si>
-    <t>Barcode händisch nachscannen</t>
-  </si>
-  <si>
     <t>Code wird manuell nachgetragen oder alternativ ein anderer Barcode-Typ (z.b. Code128) verwendet.</t>
+  </si>
+  <si>
+    <t>eine andere Vorgehensweise wird gewählt</t>
+  </si>
+  <si>
+    <t>Eine sehr genaue Tiefenkamera wurde gewählt, welche manuel auf die Anwendung kalibriert werden kann</t>
+  </si>
+  <si>
+    <t>wird nicht weiter verfolgt</t>
+  </si>
+  <si>
+    <t>Es wird stattdessen eine SD-Card mit Industrial Grade verwendet</t>
+  </si>
+  <si>
+    <t>Wägezellen werden verwendet</t>
+  </si>
+  <si>
+    <t>Idee wird nicht weiter verfolgt</t>
+  </si>
+  <si>
+    <t>Datenbank</t>
+  </si>
+  <si>
+    <t>Es werden manuelle Eingabefelder hinzugefügt. Das weitere vorgehen wird der Firma selbst überlassen</t>
   </si>
 </sst>
 </file>
@@ -315,12 +306,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -377,21 +365,16 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5C37173-CC8D-44C7-8CD7-DAA1C21A6AEA}" name="Tabelle1" displayName="Tabelle1" ref="A1:G34" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" tableBorderDxfId="7">
-  <autoFilter ref="A1:G34" xr:uid="{D5C37173-CC8D-44C7-8CD7-DAA1C21A6AEA}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{184D211B-DBE5-4DCA-965C-A9F7F7022B89}" name="Thema" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{2D4851FF-3EEE-4997-8940-9319DA4C0099}" name="Beschreibung" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{EDCF8440-BBF0-4BEB-AE53-DE814B7A7D78}" name="Priorität" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{CC79F2B8-F626-4041-A0A1-B9DF7BA39F45}" name="Eintrittswahrscheinlichkeit" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{84567F66-E4D6-486C-A0AF-52B152229E5D}" name="Auswirkung" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{803C2E62-3229-4BD4-A53E-267ABDAD66A9}" name="Umsetzung" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{9A058903-270B-433B-A361-9497577C6FD4}" name="Risikoantwort?" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5C37173-CC8D-44C7-8CD7-DAA1C21A6AEA}" name="Tabelle1" displayName="Tabelle1" ref="A1:F32" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A1:F32" xr:uid="{D5C37173-CC8D-44C7-8CD7-DAA1C21A6AEA}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{184D211B-DBE5-4DCA-965C-A9F7F7022B89}" name="Thema" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{2D4851FF-3EEE-4997-8940-9319DA4C0099}" name="Beschreibung" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{EDCF8440-BBF0-4BEB-AE53-DE814B7A7D78}" name="Priorität" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{CC79F2B8-F626-4041-A0A1-B9DF7BA39F45}" name="Eintrittswahrscheinlichkeit" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{84567F66-E4D6-486C-A0AF-52B152229E5D}" name="Auswirkung" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{803C2E62-3229-4BD4-A53E-267ABDAD66A9}" name="Risikoantwort?" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -714,19 +697,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" customWidth="1"/>
-    <col min="2" max="2" width="33.109375" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="35.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="39.88671875" customWidth="1"/>
-    <col min="6" max="6" width="23.5546875" customWidth="1"/>
-    <col min="7" max="7" width="25.88671875" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="3" max="3" width="13" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="39.85546875" customWidth="1"/>
+    <col min="6" max="6" width="27" customWidth="1"/>
+    <col min="7" max="7" width="25.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -742,513 +725,435 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2" t="s">
+      <c r="C8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="E9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="D10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="C11" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F11" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2" t="s">
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="2"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
       <c r="B19" s="2"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="2"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
       <c r="B21" s="2"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="2"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
       <c r="B23" s="2"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="2"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="2"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="2"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="2"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="2"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="2"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="2"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="2"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="2"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-    </row>
-    <row r="34" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2" t="s">
-        <v>57</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1268,16 +1173,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="dada195d-2b4c-422f-a5d1-90c4a3de233f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B16B4D4BCD437D448872317F95B506B0" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="968e47d754937c5f35b6a3a7df170301">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="dada195d-2b4c-422f-a5d1-90c4a3de233f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d3ae0215b85f957f0f511970f78bb51" ns2:_="">
     <xsd:import namespace="dada195d-2b4c-422f-a5d1-90c4a3de233f"/>
@@ -1449,6 +1344,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="dada195d-2b4c-422f-a5d1-90c4a3de233f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A1093F-D46D-4A27-8917-A2DBB49C57E7}">
   <ds:schemaRefs>
@@ -1458,22 +1363,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FAD48FE7-BCA9-4C85-A773-677E0EE23411}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="dada195d-2b4c-422f-a5d1-90c4a3de233f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286AA34-FE32-4FAA-AC16-791A5B3CAE32}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1489,4 +1378,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FAD48FE7-BCA9-4C85-A773-677E0EE23411}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="dada195d-2b4c-422f-a5d1-90c4a3de233f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>